<commit_message>
Patch data creation and training pipeline works now
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="203">
   <si>
     <t xml:space="preserve">var_name</t>
   </si>
@@ -556,6 +556,9 @@
   </si>
   <si>
     <t xml:space="preserve">1, lbd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{1:1,2:1,3:1,4:1,5:1}</t>
   </si>
   <si>
     <t xml:space="preserve">totalseg</t>
@@ -722,24 +725,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -938,312 +945,312 @@
   <dimension ref="A1:J17"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="47.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="3" style="0" width="20.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="47.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="3" style="1" width="20.17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="0" t="s">
+      <c r="D2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="n">
+      <c r="D3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>0.01</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="0" t="s">
+      <c r="D4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="0" t="s">
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="H5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="0" t="s">
+      <c r="J5" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="D6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="0" t="s">
+      <c r="D7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="0" t="s">
+      <c r="D8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="D9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="0" t="s">
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="0" t="s">
+      <c r="D11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="D12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="0" t="s">
+      <c r="D13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="0" t="s">
+      <c r="D14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="F14" s="1" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="0" t="s">
+      <c r="D15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="0" t="s">
+      <c r="D16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="0" t="s">
+      <c r="D17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1266,190 +1273,190 @@
   <dimension ref="A1:K1048576"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="24.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="0" t="s">
+      <c r="D2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="H6" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J6" s="0" t="s">
+      <c r="J6" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="K6" s="0" t="s">
+      <c r="K6" s="1" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="0" t="s">
+      <c r="D7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="I7" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="0" t="s">
+      <c r="D8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D9" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="D9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="E14" s="0" t="n">
+      <c r="E14" s="1" t="n">
         <v>192</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="0" t="n">
+      <c r="E15" s="1" t="n">
         <v>128</v>
       </c>
     </row>
@@ -1474,220 +1481,220 @@
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="0" t="s">
+      <c r="B3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="0" t="s">
+      <c r="B4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F4" s="0" t="n">
+      <c r="F4" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="1" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="0" t="s">
+      <c r="B5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F5" s="0" t="n">
+      <c r="F5" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="1" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="0" t="s">
+      <c r="B6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="F6" s="0" t="n">
+      <c r="F6" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B7" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="0" t="s">
+      <c r="B7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" s="1" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="B8" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="0" t="s">
+      <c r="B8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="G8" s="1" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="0" t="s">
+      <c r="B9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="1" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1711,101 +1718,101 @@
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="0" t="s">
+      <c r="D2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D3" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="0" t="s">
+      <c r="D3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="0" t="s">
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="D5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="0" t="s">
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="D6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="D6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1829,71 +1836,71 @@
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D4" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="0" t="s">
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="0" t="s">
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="D6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1913,1810 +1920,1860 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF38"/>
+  <dimension ref="A1:AF39"/>
   <sheetFormatPr defaultColWidth="10.16796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="14" style="0" width="20.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="41.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="24.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="13.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="13.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="22.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="23" style="0" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="14" style="1" width="20.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="41.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="24.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="13.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="13.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="22.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="23" style="1" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="P1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="R1" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="S1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="T1" s="0" t="s">
+      <c r="T1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="U1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="V1" s="0" t="s">
+      <c r="U1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="W1" s="0" t="s">
+      <c r="W1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="X1" s="0" t="s">
+      <c r="X1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="Y1" s="0" t="s">
+      <c r="Y1" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="Z1" s="0" t="s">
+      <c r="Z1" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="AA1" s="0" t="s">
+      <c r="AA1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AB1" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="AC1" s="0" t="s">
+      <c r="AB1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AD1" s="0" t="s">
+      <c r="AD1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="0" t="s">
+      <c r="AE1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AF1" s="0" t="s">
+      <c r="AF1" s="1" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="L2" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M2" s="0" t="s">
+      <c r="M2" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="S2" s="0" t="s">
+      <c r="S2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T2" s="0" t="s">
+      <c r="T2" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U2" s="0" t="s">
+      <c r="U2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V2" s="4" t="b">
+      <c r="V2" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W2" s="4" t="b">
+      <c r="W2" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L3" s="0" t="s">
+      <c r="L3" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M3" s="0" t="s">
+      <c r="M3" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="Q3" s="0" t="s">
+      <c r="Q3" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="S3" s="0" t="s">
+      <c r="S3" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T3" s="0" t="s">
+      <c r="T3" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U3" s="0" t="s">
+      <c r="U3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V3" s="4" t="b">
+      <c r="V3" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W3" s="4" t="b">
+      <c r="W3" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="J4" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="K4" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L4" s="0" t="s">
+      <c r="L4" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M4" s="0" t="s">
+      <c r="M4" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="S4" s="0" t="s">
+      <c r="S4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T4" s="0" t="s">
+      <c r="T4" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U4" s="0" t="s">
+      <c r="U4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V4" s="4" t="b">
+      <c r="V4" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W4" s="4" t="b">
+      <c r="W4" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D5" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="0" t="s">
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K5" s="0" t="s">
+      <c r="K5" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L5" s="0" t="s">
+      <c r="L5" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M5" s="0" t="s">
+      <c r="M5" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="T5" s="0" t="s">
+      <c r="T5" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U5" s="0" t="s">
+      <c r="U5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V5" s="4" t="b">
+      <c r="V5" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W5" s="4" t="b">
+      <c r="W5" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="K6" s="0" t="n">
+      <c r="K6" s="1" t="n">
         <v>192</v>
       </c>
-      <c r="L6" s="0" t="s">
+      <c r="L6" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M6" s="0" t="s">
+      <c r="M6" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="S6" s="0" t="s">
+      <c r="S6" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T6" s="0" t="s">
+      <c r="T6" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U6" s="0" t="s">
+      <c r="U6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V6" s="4" t="b">
+      <c r="V6" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W6" s="4" t="b">
+      <c r="W6" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="I7" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K7" s="0" t="s">
+      <c r="K7" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L7" s="0" t="s">
+      <c r="L7" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M7" s="0" t="s">
+      <c r="M7" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="Q7" s="0" t="s">
+      <c r="Q7" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="S7" s="0" t="n">
+      <c r="S7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="T7" s="0" t="s">
+      <c r="T7" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U7" s="0" t="s">
+      <c r="U7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V7" s="4" t="b">
+      <c r="V7" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W7" s="4" t="b">
+      <c r="W7" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="I8" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K8" s="0" t="n">
+      <c r="K8" s="1" t="n">
         <v>192</v>
       </c>
-      <c r="L8" s="0" t="s">
+      <c r="L8" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M8" s="0" t="s">
+      <c r="M8" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="Q8" s="0" t="s">
+      <c r="Q8" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="S8" s="0" t="n">
+      <c r="S8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="T8" s="0" t="s">
+      <c r="T8" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U8" s="0" t="s">
+      <c r="U8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V8" s="4" t="b">
+      <c r="V8" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W8" s="4" t="b">
+      <c r="W8" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>75</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="I9" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K9" s="0" t="n">
+      <c r="K9" s="1" t="n">
         <v>192</v>
       </c>
-      <c r="L9" s="0" t="s">
+      <c r="L9" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M9" s="0" t="s">
+      <c r="M9" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="Q9" s="0" t="s">
+      <c r="Q9" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="S9" s="0" t="n">
+      <c r="S9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="T9" s="0" t="s">
+      <c r="T9" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U9" s="0" t="s">
+      <c r="U9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V9" s="4" t="b">
+      <c r="V9" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W9" s="4" t="b">
+      <c r="W9" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B10" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="I10" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K10" s="0" t="s">
+      <c r="K10" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L10" s="0" t="s">
+      <c r="L10" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="S10" s="0" t="s">
+      <c r="S10" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T10" s="0" t="s">
+      <c r="T10" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V10" s="4" t="b">
+      <c r="V10" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W10" s="4" t="b">
+      <c r="W10" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I11" s="0" t="s">
+      <c r="I11" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="K11" s="0" t="s">
+      <c r="K11" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L11" s="0" t="s">
+      <c r="L11" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="S11" s="0" t="s">
+      <c r="S11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T11" s="0" t="s">
+      <c r="T11" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V11" s="4" t="b">
+      <c r="V11" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W11" s="4" t="b">
+      <c r="W11" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="I12" s="0" t="s">
+      <c r="I12" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K12" s="0" t="s">
+      <c r="K12" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L12" s="0" t="s">
+      <c r="L12" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="S12" s="0" t="s">
+      <c r="S12" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T12" s="0" t="s">
+      <c r="T12" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="V12" s="4" t="b">
+      <c r="V12" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W12" s="4" t="b">
+      <c r="W12" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I13" s="0" t="s">
+      <c r="I13" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="J13" s="0" t="s">
+      <c r="J13" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="M13" s="0" t="s">
+      <c r="M13" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="S13" s="0" t="s">
+      <c r="S13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T13" s="0" t="s">
+      <c r="T13" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V13" s="4" t="b">
+      <c r="V13" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W13" s="4" t="b">
+      <c r="W13" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="I14" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="K14" s="0" t="s">
+      <c r="K14" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L14" s="0" t="s">
+      <c r="L14" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="S14" s="0" t="s">
+      <c r="S14" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T14" s="0" t="s">
+      <c r="T14" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V14" s="4" t="b">
+      <c r="V14" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W14" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Z14" s="0" t="s">
+      <c r="W14" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z14" s="1" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="I15" s="0" t="s">
+      <c r="I15" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K15" s="0" t="s">
+      <c r="K15" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L15" s="0" t="s">
+      <c r="L15" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="S15" s="0" t="s">
+      <c r="S15" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T15" s="0" t="s">
+      <c r="T15" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V15" s="4" t="b">
+      <c r="V15" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W15" s="4" t="b">
+      <c r="W15" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="I16" s="0" t="s">
+      <c r="I16" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J16" s="0" t="n">
+      <c r="J16" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="S16" s="0" t="s">
+      <c r="S16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V16" s="4" t="b">
+      <c r="V16" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W16" s="4" t="b">
+      <c r="W16" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I17" s="0" t="s">
+      <c r="I17" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K17" s="0" t="s">
+      <c r="K17" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="L17" s="0" t="s">
+      <c r="L17" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="S17" s="0" t="s">
+      <c r="S17" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T17" s="0" t="s">
+      <c r="T17" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="V17" s="4" t="b">
+      <c r="V17" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W17" s="4" t="b">
+      <c r="W17" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="E18" s="0" t="s">
+      <c r="E18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="0" t="s">
+      <c r="I18" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K18" s="0" t="s">
+      <c r="K18" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L18" s="0" t="s">
+      <c r="L18" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="S18" s="0" t="s">
+      <c r="S18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T18" s="0" t="s">
+      <c r="T18" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V18" s="4" t="b">
+      <c r="V18" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W18" s="4" t="b">
+      <c r="W18" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="D19" s="0" t="n">
+      <c r="D19" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="E19" s="0" t="s">
+      <c r="E19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I19" s="0" t="s">
+      <c r="I19" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="M19" s="0" t="s">
+      <c r="M19" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="T19" s="0" t="s">
+      <c r="T19" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="V19" s="4" t="b">
+      <c r="V19" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W19" s="4" t="b">
+      <c r="W19" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B20" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" s="0" t="s">
+      <c r="B20" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="F20" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H20" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="0" t="s">
+      <c r="H20" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K20" s="0" t="s">
+      <c r="K20" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L20" s="0" t="s">
+      <c r="L20" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M20" s="0" t="s">
+      <c r="M20" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="Q20" s="0" t="s">
+      <c r="Q20" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="S20" s="0" t="s">
+      <c r="S20" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T20" s="0" t="s">
+      <c r="T20" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U20" s="0" t="s">
+      <c r="U20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V20" s="4" t="b">
+      <c r="V20" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W20" s="4" t="b">
+      <c r="W20" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D21" s="0" t="n">
+      <c r="D21" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="F21" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H21" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I21" s="0" t="s">
+      <c r="H21" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K21" s="0" t="s">
+      <c r="K21" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L21" s="0" t="s">
+      <c r="L21" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M21" s="0" t="s">
+      <c r="M21" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="Q21" s="0" t="s">
+      <c r="Q21" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="S21" s="0" t="s">
+      <c r="S21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T21" s="0" t="s">
+      <c r="T21" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U21" s="0" t="s">
+      <c r="U21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V21" s="4" t="b">
+      <c r="V21" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W21" s="4" t="b">
+      <c r="W21" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D22" s="0" t="n">
+      <c r="D22" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="F22" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H22" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I22" s="0" t="s">
+      <c r="H22" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K22" s="0" t="s">
+      <c r="K22" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L22" s="0" t="s">
+      <c r="L22" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M22" s="0" t="s">
+      <c r="M22" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="O22" s="0" t="s">
+      <c r="O22" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="Q22" s="0" t="s">
+      <c r="Q22" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="S22" s="0" t="s">
+      <c r="S22" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="T22" s="0" t="s">
+      <c r="T22" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U22" s="0" t="s">
+      <c r="U22" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V22" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="W22" s="4" t="b">
+      <c r="V22" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="W22" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D23" s="0" t="n">
+      <c r="D23" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="F23" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H23" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I23" s="0" t="s">
+      <c r="H23" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K23" s="0" t="s">
+      <c r="K23" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L23" s="0" t="s">
+      <c r="L23" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M23" s="0" t="s">
+      <c r="M23" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="O23" s="0" t="s">
+      <c r="O23" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="Q23" s="0" t="s">
+      <c r="Q23" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="S23" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T23" s="0" t="s">
+      <c r="S23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T23" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U23" s="0" t="s">
+      <c r="U23" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V23" s="4" t="b">
+      <c r="V23" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W23" s="4" t="b">
+      <c r="W23" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="H24" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="S24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T24" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V24" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W24" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B25" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C25" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="D24" s="0" t="n">
+      <c r="D25" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="H24" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I24" s="0" t="s">
+      <c r="H25" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="J24" s="0" t="s">
+      <c r="J25" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K24" s="0" t="s">
+      <c r="K25" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L24" s="0" t="s">
+      <c r="L25" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M24" s="0" t="s">
+      <c r="M25" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="O24" s="0" t="s">
+      <c r="O25" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="S24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T24" s="0" t="s">
+      <c r="S25" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T25" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U24" s="0" t="s">
+      <c r="U25" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V24" s="4" t="b">
+      <c r="V25" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W24" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="W25" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B25" s="0" t="n">
+      <c r="B26" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="S26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T26" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V26" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W26" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="T27" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V27" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W27" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AF27" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B28" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P28" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="U28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V28" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="W28" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AF28" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B29" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="S29" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T29" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="U29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V29" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W29" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AF29" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B30" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="S30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T30" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="U30" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V30" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W30" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AF30" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B31" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C25" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="D25" s="0" t="n">
+      <c r="C31" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="L31" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="S31" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T31" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="U31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V31" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W31" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AF31" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B32" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="S32" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T32" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="U32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V32" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="W32" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AF32" s="1" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="S33" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T33" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="U33" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V33" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W33" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z33" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D34" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="H25" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I25" s="0" t="s">
+      <c r="F34" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H34" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I34" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K25" s="0" t="s">
+      <c r="K34" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L25" s="0" t="s">
+      <c r="L34" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="M25" s="0" t="s">
+      <c r="M34" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="O25" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="S25" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T25" s="0" t="s">
+      <c r="Q34" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="S34" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T34" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U25" s="0" t="s">
+      <c r="U34" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V25" s="4" t="b">
+      <c r="V34" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W25" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B26" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D26" s="0" t="s">
+      <c r="W34" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B35" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H35" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>192</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q35" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="S35" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T35" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V35" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W35" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="H36" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K36" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="S36" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T36" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V36" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="W36" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Y36" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B37" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="H37" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K37" s="1" t="n">
+        <v>192</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q37" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="S37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T37" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U37" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V37" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="W37" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Y37" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B38" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="H38" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="L38" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="S38" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="T38" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="U38" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="V38" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="W38" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="I26" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="K26" s="0" t="s">
+      <c r="F39" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H39" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="K39" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L26" s="0" t="s">
+      <c r="L39" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="T26" s="0" t="s">
+      <c r="M39" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="S39" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="T39" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="U26" s="0" t="s">
+      <c r="U39" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V26" s="4" t="b">
+      <c r="V39" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W26" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF26" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B27" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D27" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="I27" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="J27" s="0" t="s">
-        <v>161</v>
-      </c>
-      <c r="K27" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="L27" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="P27" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="U27" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V27" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="W27" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF27" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B28" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D28" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="I28" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K28" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="L28" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="S28" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T28" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="U28" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V28" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W28" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF28" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B29" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D29" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="I29" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K29" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="L29" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="S29" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T29" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="U29" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V29" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W29" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF29" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B30" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="C30" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D30" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="I30" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K30" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="L30" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="O30" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="S30" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T30" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="U30" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V30" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W30" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF30" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B31" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="C31" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>181</v>
-      </c>
-      <c r="I31" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="K31" s="0" t="s">
-        <v>184</v>
-      </c>
-      <c r="L31" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="N31" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="S31" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T31" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="U31" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V31" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="W31" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF31" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>185</v>
-      </c>
-      <c r="B32" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="0" t="s">
-        <v>186</v>
-      </c>
-      <c r="D32" s="0" t="n">
-        <v>20</v>
-      </c>
-      <c r="I32" s="0" t="s">
-        <v>187</v>
-      </c>
-      <c r="K32" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="L32" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="S32" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T32" s="0" t="s">
-        <v>182</v>
-      </c>
-      <c r="U32" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V32" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W32" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Z32" s="0" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="B33" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" s="0" t="s">
-        <v>189</v>
-      </c>
-      <c r="D33" s="0" t="n">
-        <v>50</v>
-      </c>
-      <c r="F33" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="H33" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I33" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K33" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="L33" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="M33" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q33" s="0" t="s">
-        <v>190</v>
-      </c>
-      <c r="S33" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T33" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="U33" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V33" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W33" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
-        <v>188</v>
-      </c>
-      <c r="B34" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C34" s="0" t="s">
-        <v>189</v>
-      </c>
-      <c r="D34" s="0" t="n">
-        <v>50</v>
-      </c>
-      <c r="F34" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="H34" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I34" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K34" s="0" t="n">
-        <v>192</v>
-      </c>
-      <c r="L34" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="M34" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q34" s="0" t="s">
-        <v>190</v>
-      </c>
-      <c r="S34" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T34" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="U34" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V34" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W34" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
-        <v>191</v>
-      </c>
-      <c r="B35" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="D35" s="0" t="n">
-        <v>50</v>
-      </c>
-      <c r="F35" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="H35" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I35" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K35" s="0" t="n">
-        <v>128</v>
-      </c>
-      <c r="L35" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="M35" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="N35" s="0" t="s">
-        <v>194</v>
-      </c>
-      <c r="Q35" s="0" t="s">
-        <v>195</v>
-      </c>
-      <c r="S35" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T35" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="U35" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V35" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="W35" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y35" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>191</v>
-      </c>
-      <c r="B36" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="C36" s="0" t="s">
-        <v>192</v>
-      </c>
-      <c r="D36" s="0" t="n">
-        <v>100</v>
-      </c>
-      <c r="F36" s="0" t="s">
-        <v>193</v>
-      </c>
-      <c r="H36" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I36" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K36" s="0" t="n">
-        <v>192</v>
-      </c>
-      <c r="L36" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="M36" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="N36" s="0" t="s">
-        <v>194</v>
-      </c>
-      <c r="Q36" s="0" t="s">
-        <v>195</v>
-      </c>
-      <c r="S36" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T36" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="U36" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V36" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="W36" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y36" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>196</v>
-      </c>
-      <c r="B37" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" s="0" t="s">
-        <v>197</v>
-      </c>
-      <c r="D37" s="0" t="n">
-        <v>50</v>
-      </c>
-      <c r="F37" s="0" t="s">
-        <v>198</v>
-      </c>
-      <c r="H37" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I37" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K37" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="L37" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="M37" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="O37" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="S37" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="T37" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="U37" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V37" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W37" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="B38" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="D38" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="F38" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="H38" s="4" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I38" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="K38" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="L38" s="0" t="s">
-        <v>154</v>
-      </c>
-      <c r="M38" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q38" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="S38" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="T38" s="0" t="s">
-        <v>156</v>
-      </c>
-      <c r="U38" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="V38" s="4" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W38" s="4" t="b">
+      <c r="W39" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
validation grid parses entire validation set, at custom frequencies
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="model_params" sheetId="1" state="visible" r:id="rId3"/>
@@ -14,6 +14,7 @@
     <sheet name="affine3d" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="loss_params" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="plans" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="resnet" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="231">
   <si>
     <t xml:space="preserve">var_name</t>
   </si>
@@ -120,6 +121,12 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
+    <t xml:space="preserve">depth_reset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[18,10,34,50,101]</t>
+  </si>
+  <si>
     <t xml:space="preserve">optimizer</t>
   </si>
   <si>
@@ -402,6 +409,9 @@
     <t xml:space="preserve">softmax</t>
   </si>
   <si>
+    <t xml:space="preserve">include_background</t>
+  </si>
+  <si>
     <t xml:space="preserve">mnemonic</t>
   </si>
   <si>
@@ -471,9 +481,6 @@
     <t xml:space="preserve">plan_test</t>
   </si>
   <si>
-    <t xml:space="preserve">run_name</t>
-  </si>
-  <si>
     <t xml:space="preserve">periodict_test</t>
   </si>
   <si>
@@ -534,9 +541,6 @@
     <t xml:space="preserve">4, lbd</t>
   </si>
   <si>
-    <t xml:space="preserve">LITS-860</t>
-  </si>
-  <si>
     <t xml:space="preserve">70</t>
   </si>
   <si>
@@ -561,6 +565,9 @@
     <t xml:space="preserve">{1:1,2:1,3:1,4:1,5:1}</t>
   </si>
   <si>
+    <t xml:space="preserve">0.75, 0.75,0.75</t>
+  </si>
+  <si>
     <t xml:space="preserve">totalseg</t>
   </si>
   <si>
@@ -621,29 +628,108 @@
     <t xml:space="preserve">kidneys</t>
   </si>
   <si>
+    <t xml:space="preserve">no kidney labels</t>
+  </si>
+  <si>
     <t xml:space="preserve">kits21</t>
   </si>
   <si>
     <t xml:space="preserve">DS.kits21/lms</t>
   </si>
   <si>
-    <t xml:space="preserve">{1:0,2:1,3:0}</t>
+    <t xml:space="preserve">{1:0,2:1,3:1}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{1:1,2:2,3:2}</t>
   </si>
   <si>
     <t xml:space="preserve">test</t>
   </si>
   <si>
     <t xml:space="preserve">drli_short, litsmc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[ResNet3D]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ResNet3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resnet_depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[10,18,34,50,101,152]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">num_classes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spatial_dims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conv1_t_size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[3,5,7]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conv1_t_stride</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1,2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no_max_pool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shortcut_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[A,B]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">widen_factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1.0,2.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feed_forward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bias_downsample</t>
+  </si>
+  <si>
+    <t xml:space="preserve">norm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[batch,instance]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">batch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">('relu', {'inplace': True})</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pretrained</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00E+00"/>
-    <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -742,11 +828,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -942,7 +1028,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.17"/>
@@ -1015,7 +1101,7 @@
       <c r="E3" s="3" t="n">
         <v>0.01</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1092,23 +1178,17 @@
       <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>32</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="D8" s="1" t="n">
         <v>0</v>
       </c>
@@ -1121,61 +1201,67 @@
         <v>35</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="C11" s="1" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1186,49 +1272,43 @@
         <v>0</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="D14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>50</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>20</v>
+      <c r="F15" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="D16" s="1" t="n">
         <v>0</v>
@@ -1239,7 +1319,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>19</v>
@@ -1251,7 +1331,24 @@
         <v>0</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>34</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1293,7 +1390,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>6</v>
@@ -1308,34 +1405,34 @@
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>20</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>30</v>
@@ -1343,44 +1440,44 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
@@ -1389,15 +1486,15 @@
         <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>19</v>
@@ -1409,29 +1506,29 @@
         <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>0</v>
@@ -1439,14 +1536,14 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>192</v>
@@ -1454,7 +1551,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>128</v>
@@ -1496,13 +1593,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>4</v>
@@ -1513,171 +1610,171 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0</v>
@@ -1686,7 +1783,7 @@
         <v>12</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>19</v>
@@ -1734,86 +1831,86 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1832,7 +1929,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1852,12 +1949,12 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>0</v>
@@ -1865,7 +1962,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>20</v>
@@ -1873,7 +1970,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>0</v>
@@ -1884,24 +1981,32 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E7" s="4" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1920,1862 +2025,2485 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF39"/>
+  <dimension ref="A1:AG44"/>
   <sheetFormatPr defaultColWidth="10.16796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="14" style="1" width="20.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="41.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="24.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="13.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="13.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="22.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="23" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="24.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="15" style="1" width="20.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="41.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="24.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="13.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="13.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="22.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="24" style="1" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>61</v>
+        <v>145</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>143</v>
+        <v>63</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>0</v>
+        <v>146</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="AA1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="AB1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="AC1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AD1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AF1" s="1" t="s">
-        <v>149</v>
+      <c r="AG1" s="1" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>151</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K2" s="1" t="s">
         <v>153</v>
       </c>
+      <c r="E2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>154</v>
+      </c>
       <c r="L2" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>49</v>
+        <v>156</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>157</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>156</v>
+        <v>51</v>
       </c>
       <c r="U2" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V2" s="5" t="b">
+      <c r="W2" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W2" s="5" t="b">
+      <c r="X2" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>151</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N3" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" s="1" t="s">
+      <c r="R3" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U3" s="1" t="s">
+      <c r="V3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V3" s="5" t="b">
+      <c r="W3" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W3" s="5" t="b">
+      <c r="X3" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>150</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>160</v>
+        <v>152</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="S4" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="T4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T4" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="U4" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V4" s="5" t="b">
+      <c r="W4" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W4" s="5" t="b">
+      <c r="X4" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="U5" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U5" s="1" t="s">
+      <c r="V5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V5" s="5" t="b">
+      <c r="W5" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W5" s="5" t="b">
+      <c r="X5" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>151</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K6" s="1" t="n">
+        <v>153</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="L6" s="1" t="n">
         <v>192</v>
       </c>
-      <c r="L6" s="1" t="s">
-        <v>154</v>
-      </c>
       <c r="M6" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>49</v>
+        <v>156</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>157</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>156</v>
+        <v>51</v>
       </c>
       <c r="U6" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V6" s="5" t="b">
+      <c r="W6" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W6" s="5" t="b">
+      <c r="X6" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="R7" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="T7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="U7" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="S7" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U7" s="1" t="s">
+      <c r="V7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V7" s="5" t="b">
+      <c r="W7" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W7" s="5" t="b">
+      <c r="X7" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E8" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G8" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>192</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N8" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="R8" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="T8" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="U8" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K8" s="1" t="n">
-        <v>192</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M8" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="S8" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U8" s="1" t="s">
+      <c r="V8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V8" s="5" t="b">
+      <c r="W8" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W8" s="5" t="b">
+      <c r="X8" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E9" s="1" t="n">
         <v>75</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>192</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N9" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="R9" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="T9" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="U9" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K9" s="1" t="n">
-        <v>192</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="S9" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U9" s="1" t="s">
+      <c r="V9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V9" s="5" t="b">
+      <c r="W9" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W9" s="5" t="b">
+      <c r="X9" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="D10" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U10" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S10" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="V10" s="5" t="b">
+      <c r="W10" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W10" s="5" t="b">
+      <c r="X10" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>153</v>
+      <c r="D11" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>154</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S11" s="1" t="s">
-        <v>49</v>
+        <v>155</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="V11" s="5" t="b">
+        <v>51</v>
+      </c>
+      <c r="U11" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="W11" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W11" s="5" t="b">
+      <c r="X11" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="D12" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>153</v>
+      <c r="E12" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S12" s="1" t="s">
-        <v>49</v>
+        <v>155</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="V12" s="5" t="b">
+        <v>51</v>
+      </c>
+      <c r="U12" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="W12" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W12" s="5" t="b">
+      <c r="X12" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>167</v>
+      <c r="D13" s="1" t="s">
+        <v>165</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="S13" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="T13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="T13" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="V13" s="5" t="b">
+      <c r="U13" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="W13" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W13" s="5" t="b">
+      <c r="X13" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="D14" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>153</v>
+        <v>165</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>169</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S14" s="1" t="s">
-        <v>49</v>
+        <v>155</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="V14" s="5" t="b">
+        <v>51</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="W14" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W14" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Z14" s="1" t="s">
-        <v>169</v>
+      <c r="X14" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="D15" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="I15" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U15" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S15" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="V15" s="5" t="b">
+      <c r="W15" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W15" s="5" t="b">
+      <c r="X15" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="J16" s="1" t="n">
+      <c r="D16" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K16" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="S16" s="1" t="s">
+      <c r="T16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V16" s="5" t="b">
+      <c r="W16" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W16" s="5" t="b">
+      <c r="X16" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="D17" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>171</v>
+        <v>165</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S17" s="1" t="s">
-        <v>49</v>
+        <v>172</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="T17" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="V17" s="5" t="b">
+        <v>51</v>
+      </c>
+      <c r="U17" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="W17" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W17" s="5" t="b">
+      <c r="X17" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="D18" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T18" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="U18" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K18" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S18" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="T18" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="V18" s="5" t="b">
+      <c r="W18" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W18" s="5" t="b">
+      <c r="X18" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="D19" s="1" t="n">
+      <c r="D19" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E19" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I19" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="M19" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="T19" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="V19" s="5" t="b">
+      <c r="J19" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="U19" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="W19" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W19" s="5" t="b">
+      <c r="X19" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>173</v>
-      </c>
       <c r="D20" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F20" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I20" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N20" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H20" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I20" s="1" t="s">
+      <c r="R20" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="T20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U20" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K20" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q20" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="S20" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T20" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U20" s="1" t="s">
+      <c r="V20" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V20" s="5" t="b">
+      <c r="W20" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W20" s="5" t="b">
+      <c r="X20" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D21" s="1" t="n">
+      <c r="D21" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E21" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I21" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N21" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H21" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I21" s="1" t="s">
+      <c r="R21" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="T21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U21" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q21" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="S21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T21" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U21" s="1" t="s">
+      <c r="V21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V21" s="5" t="b">
+      <c r="W21" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W21" s="5" t="b">
+      <c r="X21" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D22" s="1" t="n">
+      <c r="D22" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E22" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G22" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I22" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N22" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H22" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I22" s="1" t="s">
+      <c r="P22" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="T22" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U22" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K22" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="O22" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q22" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="S22" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U22" s="1" t="s">
+      <c r="V22" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V22" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
       <c r="W22" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="X22" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D23" s="1" t="n">
+      <c r="D23" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E23" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G23" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I23" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N23" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H23" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I23" s="1" t="s">
+      <c r="P23" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="R23" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="T23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U23" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K23" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="O23" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="Q23" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="S23" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T23" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U23" s="1" t="s">
+      <c r="V23" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V23" s="5" t="b">
+      <c r="W23" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W23" s="5" t="b">
+      <c r="X23" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D24" s="1" t="n">
+      <c r="D24" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="H24" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I24" s="1" t="s">
+      <c r="I24" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P24" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="T24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U24" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K24" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M24" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="O24" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="S24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U24" s="1" t="s">
+      <c r="V24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V24" s="5" t="b">
+      <c r="W24" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W24" s="5" t="b">
+      <c r="X24" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D25" s="1" t="n">
+      <c r="D25" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E25" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="H25" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>167</v>
+      <c r="I25" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
       <c r="J25" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P25" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="S25" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T25" s="1" t="s">
-        <v>156</v>
+      <c r="T25" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="U25" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V25" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V25" s="5" t="b">
+      <c r="W25" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W25" s="5" t="b">
+      <c r="X25" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D26" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="1" t="s">
+      <c r="D26" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P26" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="T26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U26" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K26" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L26" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M26" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="O26" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="S26" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T26" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U26" s="1" t="s">
+      <c r="V26" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V26" s="5" t="b">
+      <c r="W26" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W26" s="5" t="b">
+      <c r="X26" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L27" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P27" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B27" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I27" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="T27" s="1" t="s">
-        <v>156</v>
+      <c r="T27" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="U27" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="V27" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V27" s="5" t="b">
+      <c r="W27" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W27" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF27" s="1" t="n">
-        <v>10</v>
+      <c r="X27" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>178</v>
+        <v>1</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="K28" s="1" t="s">
         <v>154</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="P28" s="1" t="s">
-        <v>180</v>
+        <v>155</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="U28" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V28" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
       <c r="W28" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF28" s="1" t="n">
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X28" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG28" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>178</v>
+        <v>2</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>158</v>
+        <v>180</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>181</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S29" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T29" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="U29" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="M29" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q29" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="V29" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V29" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
       <c r="W29" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="AF29" s="1" t="n">
-        <v>10</v>
+      <c r="X29" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG29" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B30" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="M30" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="T30" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U30" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="V30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L30" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S30" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T30" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="U30" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="V30" s="5" t="b">
+      <c r="W30" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W30" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF30" s="1" t="n">
+      <c r="X30" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG30" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>178</v>
+        <v>4</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>153</v>
+        <v>180</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>160</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="O31" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="S31" s="1" t="s">
-        <v>49</v>
+        <v>155</v>
+      </c>
+      <c r="M31" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="T31" s="1" t="s">
-        <v>183</v>
+        <v>51</v>
       </c>
       <c r="U31" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="V31" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V31" s="5" t="b">
+      <c r="W31" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W31" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF31" s="1" t="n">
+      <c r="X31" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG31" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>178</v>
+        <v>5</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="K32" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="P32" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="T32" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U32" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="L32" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="N32" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="S32" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T32" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="U32" s="1" t="s">
+      <c r="V32" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V32" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
       <c r="W32" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF32" s="1" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X32" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG32" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B33" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="O33" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B33" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="D33" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="K33" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L33" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="S33" s="1" t="s">
-        <v>49</v>
-      </c>
       <c r="T33" s="1" t="s">
-        <v>183</v>
+        <v>51</v>
       </c>
       <c r="U33" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="V33" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V33" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
       <c r="W33" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="Z33" s="1" t="s">
-        <v>169</v>
+      <c r="X33" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG33" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B34" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="B34" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" s="1" t="s">
+      <c r="E34" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="D34" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="H34" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I34" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>153</v>
-      </c>
       <c r="L34" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q34" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="S34" s="1" t="s">
-        <v>49</v>
+        <v>156</v>
       </c>
       <c r="T34" s="1" t="s">
-        <v>156</v>
+        <v>51</v>
       </c>
       <c r="U34" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="V34" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V34" s="5" t="b">
+      <c r="W34" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W34" s="5" t="b">
+      <c r="X34" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E35" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="G35" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I35" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N35" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H35" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I35" s="1" t="s">
+      <c r="R35" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="T35" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U35" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K35" s="1" t="n">
-        <v>192</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q35" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="S35" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T35" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U35" s="1" t="s">
+      <c r="V35" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V35" s="5" t="b">
+      <c r="W35" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="W35" s="5" t="b">
+      <c r="X35" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B36" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" s="1" t="s">
+      <c r="E36" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I36" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L36" s="1" t="n">
+        <v>192</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="R36" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D36" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="H36" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I36" s="1" t="s">
+      <c r="T36" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U36" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K36" s="1" t="n">
-        <v>128</v>
-      </c>
-      <c r="L36" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q36" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="S36" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T36" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U36" s="1" t="s">
+      <c r="V36" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V36" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
       <c r="W36" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y36" s="1" t="n">
-        <v>1</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X36" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="D37" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="H37" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I37" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="I37" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L37" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="R37" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="T37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U37" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K37" s="1" t="n">
-        <v>192</v>
-      </c>
-      <c r="L37" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M37" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="Q37" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="S37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T37" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U37" s="1" t="s">
+      <c r="V37" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V37" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
       <c r="W37" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="Y37" s="1" t="n">
+      <c r="X37" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z37" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B38" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="I38" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L38" s="1" t="n">
+        <v>192</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N38" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="O38" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="B38" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" s="1" t="s">
+      <c r="R38" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="D38" s="1" t="n">
-        <v>50</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="H38" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I38" s="1" t="s">
+      <c r="T38" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U38" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="K38" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L38" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M38" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="O38" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="S38" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="T38" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U38" s="1" t="s">
+      <c r="V38" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="V38" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
       <c r="W38" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
+      </c>
+      <c r="X38" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z38" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="B39" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="E39" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="G39" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="I39" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="T39" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U39" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V39" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W39" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X39" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="I40" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L40" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M40" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P40" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="T40" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U40" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V40" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W40" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X40" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B41" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I41" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L41" s="1" t="n">
+        <v>160</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P41" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="T41" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U41" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V41" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W41" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X41" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B42" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I42" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L42" s="1" t="n">
+        <v>160</v>
+      </c>
+      <c r="M42" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="N42" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P42" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="T42" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U42" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V42" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W42" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X42" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B43" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I43" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L43" s="1" t="n">
+        <v>160</v>
+      </c>
+      <c r="M43" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="P43" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="T43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="U43" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V43" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W43" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X43" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B44" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I44" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="L44" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M44" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="N44" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="R44" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="T44" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="U44" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="V44" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W44" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X44" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F39" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="H39" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="L39" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="M39" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q39" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="S39" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="T39" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="U39" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="V39" s="5" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="W39" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>0.0005</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nnunet v2 resenunet training in progress . lets see..
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="211">
   <si>
     <t xml:space="preserve">var_name</t>
   </si>
@@ -640,10 +640,10 @@
     <t xml:space="preserve">no kidney labels</t>
   </si>
   <si>
-    <t xml:space="preserve">kits21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DS.kits21/lms</t>
+    <t xml:space="preserve">kits23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DS.kits23/lms</t>
   </si>
   <si>
     <t xml:space="preserve">{1:0,2:1,3:1}</t>
@@ -1996,7 +1996,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF45"/>
+  <dimension ref="A1:AF46"/>
   <sheetFormatPr defaultColWidth="10.16796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.67"/>
@@ -4113,19 +4113,16 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="B45" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G45" s="1" t="s">
-        <v>162</v>
+        <v>204</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <v>50</v>
       </c>
       <c r="I45" s="4" t="n">
         <f aca="false">FALSE()</f>
@@ -4134,20 +4131,20 @@
       <c r="J45" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="L45" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M45" s="1" t="s">
-        <v>159</v>
+      <c r="L45" s="1" t="n">
+        <v>160</v>
+      </c>
+      <c r="M45" s="1" t="n">
+        <v>96</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="R45" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T45" s="1" t="s">
-        <v>52</v>
+      <c r="P45" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="T45" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="U45" s="1" t="s">
         <v>161</v>
@@ -4160,6 +4157,62 @@
         <v>1</v>
       </c>
       <c r="X45" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Y45" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="N46" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="R46" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="T46" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="U46" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="V46" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="W46" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="X46" s="4" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
vip_label for tracking in caseidrecorder
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="210">
   <si>
     <t xml:space="preserve">var_name</t>
   </si>
@@ -461,6 +461,9 @@
   </si>
   <si>
     <t xml:space="preserve">remapping_source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vip_label</t>
   </si>
   <si>
     <t xml:space="preserve">remapping_lbd</t>
@@ -1990,7 +1993,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF46"/>
+  <dimension ref="A1:AG46"/>
   <sheetFormatPr defaultColWidth="10.16796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.67"/>
@@ -2004,14 +2007,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="15" style="1" width="20.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="41.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="24.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="13.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="13.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="22.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="24" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="15" style="1" width="20.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="41.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="24.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="13.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="13.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="22.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="25" style="1" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2073,16 +2076,16 @@
         <v>148</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="V1" s="1" t="s">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="X1" s="1" t="s">
         <v>151</v>
@@ -2094,728 +2097,731 @@
         <v>153</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>4</v>
+        <v>154</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AC1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AD1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="AF1" s="1" t="s">
-        <v>154</v>
+      <c r="AG1" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="T2" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U2" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="V2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W2" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X2" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X2" s="5" t="b">
+      <c r="Y2" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>37</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="T3" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="U3" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U3" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="V3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W3" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X3" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X3" s="5" t="b">
+      <c r="Y3" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="T4" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="U4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="U4" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="V4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W4" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X4" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X4" s="5" t="b">
+      <c r="Y4" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="U5" s="1" t="s">
         <v>161</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W5" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X5" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X5" s="5" t="b">
+      <c r="Y5" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L6" s="1" t="n">
         <v>192</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="T6" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="U6" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U6" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="V6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W6" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X6" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X6" s="5" t="b">
+      <c r="Y6" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="U7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="V7" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R7" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="T7" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W7" s="5" t="b">
+      <c r="W7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X7" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X7" s="5" t="b">
+      <c r="Y7" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L8" s="1" t="n">
         <v>192</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R8" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="T8" s="1" t="n">
+        <v>161</v>
+      </c>
+      <c r="S8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="U8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="U8" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="V8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W8" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X8" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X8" s="5" t="b">
+      <c r="Y8" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>75</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L9" s="1" t="n">
         <v>192</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R9" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="T9" s="1" t="n">
+        <v>161</v>
+      </c>
+      <c r="S9" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="U9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="U9" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="V9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W9" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X9" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X9" s="5" t="b">
+      <c r="Y9" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>20</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T10" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U10" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U10" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="W10" s="5" t="b">
+      <c r="V10" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="X10" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X10" s="5" t="b">
+      <c r="Y10" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T11" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U11" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U11" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="W11" s="5" t="b">
+      <c r="V11" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="X11" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X11" s="5" t="b">
+      <c r="Y11" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T12" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U12" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U12" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="W12" s="5" t="b">
+      <c r="V12" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="X12" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X12" s="5" t="b">
+      <c r="Y12" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>5</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="T13" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="U13" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="U13" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="W13" s="5" t="b">
+      <c r="V13" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="X13" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X13" s="5" t="b">
+      <c r="Y13" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T14" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U14" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U14" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="W14" s="5" t="b">
+      <c r="V14" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="X14" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X14" s="5" t="b">
+      <c r="Y14" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>7</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T15" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U15" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U15" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="W15" s="5" t="b">
+      <c r="V15" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="X15" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X15" s="5" t="b">
+      <c r="Y15" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>8</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K16" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="T16" s="1" t="s">
+      <c r="U16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="W16" s="5" t="b">
+      <c r="X16" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X16" s="5" t="b">
+      <c r="Y16" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>9</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T17" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U17" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U17" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="W17" s="5" t="b">
+      <c r="V17" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="X17" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X17" s="5" t="b">
+      <c r="Y17" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>20</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T18" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="U18" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="W18" s="5" t="b">
+      <c r="V18" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="X18" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X18" s="5" t="b">
+      <c r="Y18" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>40</v>
@@ -2824,250 +2830,250 @@
         <v>20</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="U19" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="W19" s="5" t="b">
+      <c r="V19" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="X19" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X19" s="5" t="b">
+      <c r="Y19" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>37</v>
       </c>
       <c r="G20" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I20" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S20" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="U20" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V20" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I20" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L20" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N20" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R20" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T20" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U20" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V20" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W20" s="5" t="b">
+      <c r="W20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X20" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X20" s="5" t="b">
+      <c r="Y20" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E21" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G21" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I21" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S21" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="U21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V21" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I21" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R21" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T21" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U21" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V21" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W21" s="5" t="b">
+      <c r="W21" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X21" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X21" s="5" t="b">
+      <c r="Y21" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G22" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I22" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="S22" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="U22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V22" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I22" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L22" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N22" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P22" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="R22" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V22" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W22" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="W22" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="X22" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Y22" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G23" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I23" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q23" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="S23" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="U23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="V23" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I23" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="R23" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T23" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U23" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V23" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W23" s="5" t="b">
+      <c r="W23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X23" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X23" s="5" t="b">
+      <c r="Y23" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>5</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>50</v>
@@ -3077,47 +3083,47 @@
         <v>0</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P24" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="T24" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U24" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="Q24" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="U24" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V24" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W24" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X24" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X24" s="5" t="b">
+      <c r="Y24" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E25" s="1" t="n">
         <v>20</v>
@@ -3127,50 +3133,50 @@
         <v>0</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K25" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="L25" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q25" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="L25" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P25" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="T25" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U25" s="1" t="s">
-        <v>161</v>
+      <c r="U25" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="V25" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W25" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W25" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X25" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X25" s="5" t="b">
+      <c r="Y25" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>7</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E26" s="1" t="n">
         <v>0</v>
@@ -3180,47 +3186,47 @@
         <v>0</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P26" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="T26" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U26" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="Q26" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="U26" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V26" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W26" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W26" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X26" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X26" s="5" t="b">
+      <c r="Y26" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>8</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>0</v>
@@ -3230,569 +3236,569 @@
         <v>0</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L27" s="1" t="n">
         <v>96</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P27" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="T27" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U27" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q27" s="1" t="s">
         <v>182</v>
       </c>
+      <c r="U27" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V27" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W27" s="5" t="b">
+        <v>183</v>
+      </c>
+      <c r="W27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X27" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X27" s="5" t="b">
+      <c r="Y27" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="U28" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="V28" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W28" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W28" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X28" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X28" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF28" s="1" t="n">
+      <c r="Y28" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG28" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>44</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q29" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="V29" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W29" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>160</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="W29" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="X29" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="AF29" s="1" t="n">
+      <c r="Y29" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG29" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T30" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U30" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U30" s="1" t="s">
-        <v>186</v>
-      </c>
       <c r="V30" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W30" s="5" t="b">
+        <v>187</v>
+      </c>
+      <c r="W30" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X30" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X30" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF30" s="1" t="n">
+      <c r="Y30" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG30" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T31" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U31" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U31" s="1" t="s">
-        <v>188</v>
-      </c>
       <c r="V31" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W31" s="5" t="b">
+        <v>189</v>
+      </c>
+      <c r="W31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X31" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X31" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF31" s="1" t="n">
+      <c r="Y31" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG31" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>5</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="P32" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="U32" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V32" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="T32" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U32" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="V32" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W32" s="5" t="b">
+      <c r="W32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X32" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X32" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AF32" s="1" t="n">
+      <c r="Y32" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG32" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L33" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="O33" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="M33" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="O33" s="1" t="s">
+      <c r="U33" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V33" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="T33" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U33" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="V33" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W33" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+      <c r="W33" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="X33" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="AF33" s="1" t="n">
+      <c r="Y33" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="AG33" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E34" s="1" t="n">
         <v>20</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="T34" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="U34" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U34" s="1" t="s">
-        <v>188</v>
-      </c>
       <c r="V34" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W34" s="5" t="b">
+        <v>189</v>
+      </c>
+      <c r="W34" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X34" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X34" s="5" t="b">
+      <c r="Y34" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E35" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G35" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I35" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M35" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N35" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S35" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="U35" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V35" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I35" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L35" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M35" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N35" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R35" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="T35" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U35" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V35" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W35" s="5" t="b">
+      <c r="W35" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X35" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X35" s="5" t="b">
+      <c r="Y35" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E36" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I36" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L36" s="1" t="n">
         <v>192</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R36" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="T36" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S36" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="U36" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="U36" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="V36" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W36" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X36" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X36" s="5" t="b">
+      <c r="Y36" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I37" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L37" s="1" t="n">
         <v>128</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="R37" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="T37" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U37" s="1" t="s">
-        <v>161</v>
+      <c r="S37" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="U37" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="V37" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W37" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>162</v>
+      </c>
+      <c r="W37" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="X37" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Y37" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E38" s="1" t="n">
         <v>100</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I38" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L38" s="1" t="n">
         <v>192</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="R38" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="T38" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U38" s="1" t="s">
-        <v>161</v>
+      <c r="S38" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="U38" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="V38" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W38" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>162</v>
+      </c>
+      <c r="W38" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="X38" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Y38" s="5" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E39" s="1" t="n">
         <v>50</v>
@@ -3802,7 +3808,7 @@
         <v>0</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L39" s="1" t="n">
         <v>160</v>
@@ -3811,38 +3817,41 @@
         <v>96</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="T39" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U39" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="P39" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="U39" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V39" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W39" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="W39" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X39" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X39" s="4" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y39" s="1" t="n">
+      <c r="Y39" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z39" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E40" s="1" t="n">
         <v>50</v>
@@ -3852,50 +3861,53 @@
         <v>0</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P40" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="T40" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U40" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="P40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q40" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="U40" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V40" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W40" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W40" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X40" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X40" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y40" s="1" t="n">
+      <c r="Y40" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z40" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E41" s="1" t="n">
         <v>100</v>
@@ -3905,50 +3917,53 @@
         <v>0</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L41" s="1" t="n">
         <v>160</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P41" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="T41" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U41" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="P41" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q41" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="U41" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V41" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W41" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W41" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X41" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X41" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y41" s="1" t="n">
+      <c r="Y41" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z41" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>4</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E42" s="1" t="n">
         <v>100</v>
@@ -3958,7 +3973,7 @@
         <v>0</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L42" s="1" t="n">
         <v>160</v>
@@ -3967,41 +3982,44 @@
         <v>64</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P42" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="T42" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U42" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="P42" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="U42" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V42" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W42" s="5" t="b">
+        <v>162</v>
+      </c>
+      <c r="W42" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X42" s="5" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X42" s="5" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y42" s="1" t="n">
+      <c r="Y42" s="5" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z42" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>5</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E43" s="1" t="n">
         <v>100</v>
@@ -4011,7 +4029,7 @@
         <v>0</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L43" s="1" t="n">
         <v>160</v>
@@ -4020,41 +4038,44 @@
         <v>64</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P43" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="T43" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U43" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="P43" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="U43" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V43" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W43" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="W43" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X43" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X43" s="4" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y43" s="1" t="n">
+      <c r="Y43" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z43" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B44" s="1" t="n">
         <v>6</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E44" s="1" t="n">
         <v>20</v>
@@ -4064,7 +4085,7 @@
         <v>0</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L44" s="1" t="n">
         <v>160</v>
@@ -4073,41 +4094,44 @@
         <v>96</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P44" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="T44" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U44" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="P44" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q44" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="U44" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V44" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W44" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="W44" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X44" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X44" s="4" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y44" s="1" t="n">
+      <c r="Y44" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z44" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B45" s="1" t="n">
         <v>7</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E45" s="1" t="n">
         <v>50</v>
@@ -4117,7 +4141,7 @@
         <v>0</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L45" s="1" t="n">
         <v>160</v>
@@ -4126,81 +4150,84 @@
         <v>96</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="P45" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="T45" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="U45" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="P45" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q45" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="U45" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="V45" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W45" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="W45" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X45" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X45" s="4" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="Y45" s="1" t="n">
+      <c r="Y45" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z45" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B46" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>37</v>
       </c>
       <c r="G46" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N46" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S46" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="U46" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V46" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="I46" s="4" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L46" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="M46" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="N46" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="R46" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="T46" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="U46" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="V46" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="W46" s="4" t="n">
+      <c r="W46" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X46" s="4" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="X46" s="4" t="n">
+      <c r="Y46" s="4" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4283,7 +4310,7 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="I8" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
sliding window hooked to case recorder wandb and seems to work
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="211">
   <si>
     <t xml:space="preserve">var_name</t>
   </si>
@@ -647,6 +647,9 @@
   </si>
   <si>
     <t xml:space="preserve">{1:1,2:2,3:2}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.8,.8,0.8</t>
   </si>
   <si>
     <t xml:space="preserve">test</t>
@@ -1993,7 +1996,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AG46"/>
+  <dimension ref="A1:AG47"/>
   <sheetFormatPr defaultColWidth="10.16796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.67"/>
@@ -4178,19 +4181,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B46" s="1" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G46" s="1" t="s">
-        <v>163</v>
+        <v>205</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>50</v>
       </c>
       <c r="I46" s="4" t="n">
         <f aca="false">FALSE()</f>
@@ -4199,23 +4199,26 @@
       <c r="J46" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="L46" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="M46" s="1" t="s">
-        <v>160</v>
+      <c r="L46" s="1" t="n">
+        <v>192</v>
+      </c>
+      <c r="M46" s="1" t="n">
+        <v>128</v>
       </c>
       <c r="N46" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="S46" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="U46" s="1" t="s">
-        <v>52</v>
+      <c r="P46" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q46" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="U46" s="1" t="n">
+        <v>1</v>
       </c>
       <c r="V46" s="1" t="s">
-        <v>162</v>
+        <v>207</v>
       </c>
       <c r="W46" s="1" t="s">
         <v>4</v>
@@ -4225,6 +4228,62 @@
         <v>1</v>
       </c>
       <c r="Y46" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="Z46" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L47" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M47" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="N47" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="S47" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="U47" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V47" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="W47" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="X47" s="4" t="n">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="Y47" s="4" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
@@ -4307,7 +4366,7 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="I8" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
fixed_spacing aligned to labelbounded.py
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="213">
   <si>
     <t xml:space="preserve">var_name</t>
   </si>
@@ -655,7 +655,13 @@
     <t xml:space="preserve">test</t>
   </si>
   <si>
-    <t xml:space="preserve">drli_short, litsmc</t>
+    <t xml:space="preserve">drli_short, lidc_short,kits23_short</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{1:0,2:1,3:1},{1:1,2:1,3:2,4:2,5:2},{1:1,2:2,3:2}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSL.label_localiser:TSL.lungs,None,None</t>
   </si>
   <si>
     <t xml:space="preserve">\</t>
@@ -2010,7 +2016,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="15" style="1" width="20.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="20.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="13.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="14.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="20.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="41.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="24.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="8.67"/>
@@ -4267,8 +4276,11 @@
       <c r="N47" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="O47" s="1" t="s">
+        <v>210</v>
+      </c>
       <c r="S47" s="1" t="s">
-        <v>179</v>
+        <v>211</v>
       </c>
       <c r="U47" s="1" t="s">
         <v>52</v>
@@ -4366,7 +4378,7 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="I8" s="6" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
bugfs in whole data trainer
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -686,13 +686,13 @@
     <t xml:space="preserve">test</t>
   </si>
   <si>
-    <t xml:space="preserve">drli_short, lidc_short,kits23_short</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{1:0,2:1,3:1},{1:1,2:1,3:2,4:2,5:2},{1:1,2:2,3:2}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TSL.label_region:TSL.lungs,None,None</t>
+    <t xml:space="preserve">drli_short, lidc_short,kits23_short,nodes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{1:0,2:1,3:1},{1:1,2:1,3:2,4:2,5:2},{1:1,2:2,3:2},None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSL.label_region:TSL.lungs,None,None,None</t>
   </si>
   <si>
     <t xml:space="preserve">[ResNet3D]</t>
@@ -2145,7 +2145,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="38.21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="8.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="8.67"/>

</xml_diff>

<commit_message>
yolo2 to become yolo.py and delete cascade_yolo.py
</commit_message>
<xml_diff>
--- a/configurations/experiment_configs.xlsx
+++ b/configurations/experiment_configs.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="231">
   <si>
     <t xml:space="preserve">var_name</t>
   </si>
@@ -596,6 +596,9 @@
     <t xml:space="preserve">192</t>
   </si>
   <si>
+    <t xml:space="preserve">all</t>
+  </si>
+  <si>
     <t xml:space="preserve">rbd</t>
   </si>
   <si>
@@ -641,7 +644,7 @@
     <t xml:space="preserve">kits23</t>
   </si>
   <si>
-    <t xml:space="preserve">abdomen, pelvis</t>
+    <t xml:space="preserve">abdomen</t>
   </si>
   <si>
     <t xml:space="preserve">all labels, abdomen lbd</t>
@@ -672,9 +675,6 @@
   </si>
   <si>
     <t xml:space="preserve">totalseg_short</t>
-  </si>
-  <si>
-    <t xml:space="preserve">all</t>
   </si>
   <si>
     <t xml:space="preserve">[ResNet3D]</t>
@@ -3554,8 +3554,11 @@
       <c r="E31" s="1" t="n">
         <v>10</v>
       </c>
+      <c r="I31" s="1" t="s">
+        <v>189</v>
+      </c>
       <c r="J31" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="L31" s="1" t="s">
         <v>188</v>
@@ -3589,19 +3592,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E32" s="1" t="n">
         <v>20</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>157</v>
@@ -3629,13 +3632,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E33" s="1" t="n">
         <v>50</v>
@@ -3660,7 +3663,7 @@
         <v>159</v>
       </c>
       <c r="R33" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="V33" s="4" t="s">
         <v>50</v>
@@ -3682,13 +3685,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E34" s="1" t="n">
         <v>50</v>
@@ -3713,7 +3716,7 @@
         <v>159</v>
       </c>
       <c r="R34" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="V34" s="4" t="s">
         <v>50</v>
@@ -3735,19 +3738,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E35" s="1" t="n">
         <v>50</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H35" s="6" t="b">
         <f aca="false">FALSE()</f>
@@ -3766,10 +3769,10 @@
         <v>159</v>
       </c>
       <c r="O35" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="R35" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="V35" s="1" t="n">
         <v>1</v>
@@ -3791,19 +3794,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E36" s="1" t="n">
         <v>100</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H36" s="6" t="b">
         <f aca="false">FALSE()</f>
@@ -3822,10 +3825,10 @@
         <v>159</v>
       </c>
       <c r="O36" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="R36" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="V36" s="1" t="n">
         <v>1</v>
@@ -3847,16 +3850,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E37" s="1" t="n">
         <v>50</v>
@@ -3900,13 +3903,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E38" s="1" t="n">
         <v>0</v>
@@ -3916,10 +3919,10 @@
         <v>0</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="L38" s="1" t="n">
         <v>160</v>
@@ -3953,16 +3956,16 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>9</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E39" s="1" t="n">
         <v>50</v>
@@ -3987,7 +3990,7 @@
         <v>159</v>
       </c>
       <c r="R39" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="T39" s="1" t="n">
         <v>3</v>
@@ -4012,13 +4015,13 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>35</v>
@@ -4040,10 +4043,10 @@
         <v>64</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="V40" s="4" t="s">
         <v>50</v>
@@ -4065,13 +4068,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>35</v>
@@ -4093,10 +4096,10 @@
         <v>96</v>
       </c>
       <c r="O41" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="R41" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="V41" s="4" t="s">
         <v>50</v>
@@ -4118,23 +4121,23 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>35</v>
       </c>
       <c r="H42" s="5"/>
       <c r="I42" s="1" t="s">
-        <v>215</v>
+        <v>189</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="L42" s="1" t="n">
         <v>160</v>
@@ -4430,13 +4433,13 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>226</v>

</xml_diff>